<commit_message>
updated model, much simpler
</commit_message>
<xml_diff>
--- a/results_diabetes_korea.xlsx
+++ b/results_diabetes_korea.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI3"/>
+  <dimension ref="A1:AF3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -427,105 +427,90 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>p_t1_med</t>
+          <t>PAF_med</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>p_t2_med</t>
+          <t>PAF_lo</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>p_t3_med</t>
+          <t>PAF_hi</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>PAF_med</t>
+          <t>AC_med</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>PAF_lo</t>
+          <t>AC_lo</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>PAF_hi</t>
+          <t>AC_hi</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>AC_med</t>
+          <t>AD_med</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>AC_lo</t>
+          <t>AD_lo</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>AC_hi</t>
+          <t>AD_hi</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>AD_med</t>
+          <t>YLD_med</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>AD_lo</t>
+          <t>YLD_lo</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>AD_hi</t>
+          <t>YLD_hi</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>YLD_med</t>
+          <t>YLL_med</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>YLD_lo</t>
+          <t>YLL_lo</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>YLD_hi</t>
+          <t>YLL_hi</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>YLL_med</t>
+          <t>DALY_med</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>YLL_lo</t>
+          <t>DALY_lo</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>YLL_hi</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>DALY_med</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>DALY_lo</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>DALY_hi</t>
         </is>
@@ -574,70 +559,61 @@
         <v>13.82599798902785</v>
       </c>
       <c r="N2">
-        <v>0.9384</v>
+        <v>0.9385</v>
       </c>
       <c r="O2">
-        <v>0.06420648961108927</v>
+        <v>0.4697196200574989</v>
       </c>
       <c r="P2">
-        <v>0.1617177516201753</v>
+        <v>0.1839933540414108</v>
       </c>
       <c r="Q2">
-        <v>0.7740612508104384</v>
+        <v>0.6500952158769256</v>
       </c>
       <c r="R2">
-        <v>0.4703568805147512</v>
+        <v>3689.647615551654</v>
       </c>
       <c r="S2">
-        <v>0.2464449720719331</v>
+        <v>1445.267795995281</v>
       </c>
       <c r="T2">
-        <v>0.6336240182442978</v>
+        <v>5106.497920713252</v>
       </c>
       <c r="U2">
-        <v>3694.653296443371</v>
+        <v>266.2793554143956</v>
       </c>
       <c r="V2">
-        <v>1935.825255625034</v>
+        <v>104.3039924725353</v>
       </c>
       <c r="W2">
-        <v>4977.116663308959</v>
+        <v>368.5324769284704</v>
       </c>
       <c r="X2">
-        <v>266.6406119950073</v>
+        <v>3271.689610941363</v>
       </c>
       <c r="Y2">
-        <v>139.7071902178581</v>
+        <v>1216.649754297117</v>
       </c>
       <c r="Z2">
-        <v>359.1951197025099</v>
+        <v>5197.782828117713</v>
       </c>
       <c r="AA2">
-        <v>3266.801729774726</v>
+        <v>3681.577832479066</v>
       </c>
       <c r="AB2">
-        <v>1687.124064179943</v>
+        <v>1442.10679017285</v>
       </c>
       <c r="AC2">
-        <v>5018.111615461413</v>
+        <v>5095.329284904486</v>
       </c>
       <c r="AD2">
-        <v>3686.572565236127</v>
+        <v>7012.954283952877</v>
       </c>
       <c r="AE2">
-        <v>1931.591331004838</v>
+        <v>2660.64412899774</v>
       </c>
       <c r="AF2">
-        <v>4966.231002675522</v>
-      </c>
-      <c r="AG2">
-        <v>6991.882734637303</v>
-      </c>
-      <c r="AH2">
-        <v>3709.305075063096</v>
-      </c>
-      <c r="AI2">
-        <v>9803.633669365789</v>
+        <v>10041.58840446876</v>
       </c>
     </row>
     <row r="3">
@@ -683,70 +659,61 @@
         <v>17.75734615707216</v>
       </c>
       <c r="N3">
-        <v>0.9752</v>
+        <v>0.9751</v>
       </c>
       <c r="O3">
-        <v>0.04132061929662668</v>
+        <v>0.4994597125555089</v>
       </c>
       <c r="P3">
-        <v>0.1390171334769673</v>
+        <v>0.2054538027565726</v>
       </c>
       <c r="Q3">
-        <v>0.8195863022978248</v>
+        <v>0.6933002655526372</v>
       </c>
       <c r="R3">
-        <v>0.4941464000956235</v>
+        <v>5327.237294117058</v>
       </c>
       <c r="S3">
-        <v>0.2452609588962506</v>
+        <v>2191.370260201603</v>
       </c>
       <c r="T3">
-        <v>0.6681096979214923</v>
+        <v>7394.740632384429</v>
       </c>
       <c r="U3">
-        <v>5270.565503419921</v>
+        <v>357.2835107794577</v>
       </c>
       <c r="V3">
-        <v>2615.953387587409</v>
+        <v>146.9693232638867</v>
       </c>
       <c r="W3">
-        <v>7126.058038030636</v>
+        <v>495.9454119604235</v>
       </c>
       <c r="X3">
-        <v>353.4826858444034</v>
+        <v>4347.550264149384</v>
       </c>
       <c r="Y3">
-        <v>175.4449743368439</v>
+        <v>1738.03385837933</v>
       </c>
       <c r="Z3">
-        <v>477.9255913111604</v>
+        <v>6940.325448327808</v>
       </c>
       <c r="AA3">
-        <v>4276.31571092201</v>
+        <v>6344.406977124856</v>
       </c>
       <c r="AB3">
-        <v>2062.579530260443</v>
+        <v>2609.785147667475</v>
       </c>
       <c r="AC3">
-        <v>6671.525693861908</v>
+        <v>8806.674355192999</v>
       </c>
       <c r="AD3">
-        <v>6276.914413070663</v>
+        <v>10761.21635823929</v>
       </c>
       <c r="AE3">
-        <v>3115.43714081798</v>
+        <v>4406.879697828529</v>
       </c>
       <c r="AF3">
-        <v>8486.690162235675</v>
-      </c>
-      <c r="AG3">
-        <v>10562.76031628667</v>
-      </c>
-      <c r="AH3">
-        <v>5254.263516507257</v>
-      </c>
-      <c r="AI3">
-        <v>14806.21075306504</v>
+        <v>15391.79314315575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
name fix and upload of excel
</commit_message>
<xml_diff>
--- a/results_diabetes_korea.xlsx
+++ b/results_diabetes_korea.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF3"/>
+  <dimension ref="A1:AH3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -407,110 +407,120 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>p_detectable_dk</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>mean_exp_dk</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>median_dk</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>D_years</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>deaths</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>seyll</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>p_detectable_med</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>PAF_med</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>PAF_lo</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>PAF_hi</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>AC_med</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>AC_lo</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>AC_hi</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>AD_med</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>AD_lo</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>AD_hi</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>YLD_med</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>YLD_lo</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>YLD_hi</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>YLL_med</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>YLL_lo</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>YLL_hi</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>DALY_med</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>DALY_lo</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>DALY_hi</t>
         </is>
@@ -550,70 +560,76 @@
         <v>1.459948535832434</v>
       </c>
       <c r="K2">
+        <v>0.938467460514304</v>
+      </c>
+      <c r="L2">
+        <v>0.5515590672171771</v>
+      </c>
+      <c r="M2">
+        <v>0.19</v>
+      </c>
+      <c r="N2">
         <v>18.2</v>
       </c>
-      <c r="L2">
+      <c r="O2">
         <v>566.89</v>
       </c>
-      <c r="M2">
+      <c r="P2">
         <v>13.82599798902785</v>
       </c>
-      <c r="N2">
-        <v>0.9385</v>
-      </c>
-      <c r="O2">
-        <v>0.4697196200574989</v>
-      </c>
-      <c r="P2">
-        <v>0.1839933540414108</v>
-      </c>
       <c r="Q2">
-        <v>0.6500952158769256</v>
+        <v>0.6769554448593391</v>
       </c>
       <c r="R2">
-        <v>3689.647615551654</v>
+        <v>0.3254537890667784</v>
       </c>
       <c r="S2">
-        <v>1445.267795995281</v>
+        <v>0.8256437760794945</v>
       </c>
       <c r="T2">
-        <v>5106.497920713252</v>
+        <v>5317.48501937011</v>
       </c>
       <c r="U2">
-        <v>266.2793554143956</v>
+        <v>2556.439513119544</v>
       </c>
       <c r="V2">
-        <v>104.3039924725353</v>
+        <v>6485.431861104429</v>
       </c>
       <c r="W2">
-        <v>368.5324769284704</v>
+        <v>383.7592721363108</v>
       </c>
       <c r="X2">
-        <v>3271.689610941363</v>
+        <v>184.496498484066</v>
       </c>
       <c r="Y2">
-        <v>1216.649754297117</v>
+        <v>468.0492002217046</v>
       </c>
       <c r="Z2">
-        <v>5197.782828117713</v>
+        <v>4623.789535271488</v>
       </c>
       <c r="AA2">
-        <v>3681.577832479066</v>
+        <v>2163.189482566324</v>
       </c>
       <c r="AB2">
-        <v>1442.10679017285</v>
+        <v>6912.804310593957</v>
       </c>
       <c r="AC2">
-        <v>5095.329284904486</v>
+        <v>5305.854924827427</v>
       </c>
       <c r="AD2">
-        <v>7012.954283952877</v>
+        <v>2550.848217023377</v>
       </c>
       <c r="AE2">
-        <v>2660.64412899774</v>
+        <v>6471.247301031383</v>
       </c>
       <c r="AF2">
-        <v>10041.58840446876</v>
+        <v>9959.374027093705</v>
+      </c>
+      <c r="AG2">
+        <v>4886.106346788335</v>
+      </c>
+      <c r="AH2">
+        <v>13063.45916041361</v>
       </c>
     </row>
     <row r="3">
@@ -650,70 +666,76 @@
         <v>1.222152467927124</v>
       </c>
       <c r="K3">
+        <v>0.9751202882482998</v>
+      </c>
+      <c r="L3">
+        <v>0.4642651689432709</v>
+      </c>
+      <c r="M3">
+        <v>0.22</v>
+      </c>
+      <c r="N3">
         <v>16.7</v>
       </c>
-      <c r="L3">
+      <c r="O3">
         <v>715.34</v>
       </c>
-      <c r="M3">
+      <c r="P3">
         <v>17.75734615707216</v>
       </c>
-      <c r="N3">
-        <v>0.9751</v>
-      </c>
-      <c r="O3">
-        <v>0.4994597125555089</v>
-      </c>
-      <c r="P3">
-        <v>0.2054538027565726</v>
-      </c>
       <c r="Q3">
-        <v>0.6933002655526372</v>
+        <v>0.751569512307089</v>
       </c>
       <c r="R3">
-        <v>5327.237294117058</v>
+        <v>0.4166166691376174</v>
       </c>
       <c r="S3">
-        <v>2191.370260201603</v>
+        <v>0.8938962471122412</v>
       </c>
       <c r="T3">
-        <v>7394.740632384429</v>
+        <v>8016.240418267412</v>
       </c>
       <c r="U3">
-        <v>357.2835107794577</v>
+        <v>4443.633393021827</v>
       </c>
       <c r="V3">
-        <v>146.9693232638867</v>
+        <v>9534.297371699164</v>
       </c>
       <c r="W3">
-        <v>495.9454119604235</v>
+        <v>537.6277349337531</v>
       </c>
       <c r="X3">
-        <v>4347.550264149384</v>
+        <v>298.0225681009033</v>
       </c>
       <c r="Y3">
-        <v>1738.03385837933</v>
+        <v>639.4397414092707</v>
       </c>
       <c r="Z3">
-        <v>6940.325448327808</v>
+        <v>6408.597720447829</v>
       </c>
       <c r="AA3">
-        <v>6344.406977124856</v>
+        <v>3222.593943830894</v>
       </c>
       <c r="AB3">
-        <v>2609.785147667475</v>
+        <v>9392.546495758741</v>
       </c>
       <c r="AC3">
-        <v>8806.674355192999</v>
+        <v>9546.841792861291</v>
       </c>
       <c r="AD3">
-        <v>10761.21635823929</v>
+        <v>5292.089904387351</v>
       </c>
       <c r="AE3">
-        <v>4406.879697828529</v>
+        <v>11354.75283479313</v>
       </c>
       <c r="AF3">
-        <v>15391.79314315575</v>
+        <v>16002.5520766779</v>
+      </c>
+      <c r="AG3">
+        <v>8760.869428147402</v>
+      </c>
+      <c r="AH3">
+        <v>20264.08520885761</v>
       </c>
     </row>
   </sheetData>

</xml_diff>